<commit_message>
Comitting & pushing for backup purposes
</commit_message>
<xml_diff>
--- a/Time_Tracking/WorkHours_Calculator_2026.xlsx
+++ b/Time_Tracking/WorkHours_Calculator_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\Time_Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ED4C3BC-C0BA-4F10-9879-F99257C5134E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548AA828-23CB-42F5-B71A-E6ED1F2E67F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39690" yWindow="1470" windowWidth="31365" windowHeight="15345" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
+    <workbookView xWindow="2565" yWindow="1365" windowWidth="31365" windowHeight="15345" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
   </bookViews>
   <sheets>
     <sheet name="20260921" sheetId="38" r:id="rId1"/>
@@ -4790,35 +4790,39 @@
       <c r="B3" s="8">
         <v>0.28819444444444442</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+      <c r="C3" s="8">
+        <v>0.5625</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0.59444444444444444</v>
+      </c>
       <c r="E3" s="8">
         <v>0.66666666666666663</v>
       </c>
       <c r="F3" s="30">
         <f t="shared" ref="F3:F6" si="0">IF(G3 &gt;= 8, 4 + COUNT(B3:E3), IF(AND(G3 &gt;= 4, G3 &lt;= 7), 2 + COUNT(B3:E3), COUNT(B3:E3)))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3" s="28"/>
       <c r="H3" s="10">
         <f>SUM(C3 - B3) * 24</f>
-        <v>-6.9166666666666661</v>
+        <v>6.5833333333333339</v>
       </c>
       <c r="I3" s="11">
         <f>SUM(E3 - D3) * 24</f>
-        <v>16</v>
+        <v>1.7333333333333325</v>
       </c>
       <c r="J3" s="12">
         <f t="shared" ref="J3:J6" si="1">H3 + I3 + G3</f>
-        <v>9.0833333333333339</v>
-      </c>
-      <c r="K3" s="13" t="str">
+        <v>8.3166666666666664</v>
+      </c>
+      <c r="K3" s="13">
         <f>IF(AND(C3 &lt;&gt; "", D3 &lt;&gt; ""), (SUM(D3 - C3) * 1440), " - ")</f>
-        <v xml:space="preserve"> - </v>
-      </c>
-      <c r="L3" s="14" t="str">
+        <v>46</v>
+      </c>
+      <c r="L3" s="14">
         <f>IF(AND((B3 &lt;&gt; ""), (C3 &lt;&gt; ""), (D3 &lt;&gt; ""), (E3 &lt;&gt; "")), IF((((8 - J3) * 60) + 1) &gt; 0, (((8 - J3) * 60) + 1), (((8 - J3) * 60) - 1)), "-")</f>
-        <v>-</v>
+        <v>-19.999999999999986</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -4826,34 +4830,42 @@
         <f ca="1">_xlfn.CONCAT(TEXT(A1 + 2, "ddd"), " (", DAY(A1 + 2), IF(OR(AND(DAY(A1 + 2) &gt; 23, DAY(A1 + 2) &lt; 31), AND(DAY(A1 + 2) &gt; 3, DAY(A1 + 2) &lt; 21)), "th", LOOKUP(DAY(A1 + 2), {1,"st";2,"nd";3,"rd";21,"st";22,"nd";23,"rd";31,"st"})), ")")</f>
         <v>Wed (23rd)</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
+      <c r="B4" s="8">
+        <v>0.28819444444444442</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.58194444444444449</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.61319444444444449</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F4" s="30">
         <f>IF(G4 &gt;= 8, 4 + COUNT(B4:E4), IF(AND(G4 &gt;= 4, G4 &lt;= 7), 2 + COUNT(B4:E4), COUNT(B4:E4)))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G4" s="28"/>
       <c r="H4" s="10">
         <f t="shared" ref="H4:H5" si="2">SUM(C4 - B4) * 24</f>
-        <v>0</v>
+        <v>7.0500000000000016</v>
       </c>
       <c r="I4" s="11">
         <f t="shared" ref="I4:I6" si="3">SUM(E4 - D4) * 24</f>
-        <v>0</v>
+        <v>1.2833333333333314</v>
       </c>
       <c r="J4" s="12">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K4" s="13" t="str">
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="K4" s="13">
         <f t="shared" ref="K4:K6" si="4">IF(AND(C4 &lt;&gt; "", D4 &lt;&gt; ""), (SUM(D4 - C4) * 1440), " - ")</f>
-        <v xml:space="preserve"> - </v>
-      </c>
-      <c r="L4" s="14" t="str">
+        <v>45</v>
+      </c>
+      <c r="L4" s="14">
         <f t="shared" ref="L4:L5" si="5">IF(AND((B4 &lt;&gt; ""), (C4 &lt;&gt; ""), (D4 &lt;&gt; ""), (E4 &lt;&gt; "")), IF((((8 - J4) * 60) + 1) &gt; 0, (((8 - J4) * 60) + 1), (((8 - J4) * 60) - 1)), "-")</f>
-        <v>-</v>
+        <v>-20.999999999999929</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -4861,26 +4873,32 @@
         <f ca="1">_xlfn.CONCAT(TEXT(A1 + 3, "ddd"), " (", DAY(A1 + 3), IF(OR(AND(DAY(A1 + 3) &gt; 23, DAY(A1 + 3) &lt; 31), AND(DAY(A1 + 3) &gt; 3, DAY(A1 + 3) &lt; 21)), "th", LOOKUP(DAY(A1 + 3), {1,"st";2,"nd";3,"rd";21,"st";22,"nd";23,"rd";31,"st"})), ")")</f>
         <v>Thu (24th)</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
+      <c r="B5" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="8">
+        <v>0.54166666666666663</v>
+      </c>
       <c r="F5" s="30">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="28"/>
+        <v>4</v>
+      </c>
+      <c r="G5" s="28">
+        <v>4</v>
+      </c>
       <c r="H5" s="10">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-9</v>
       </c>
       <c r="I5" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J5" s="12">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K5" s="13" t="str">
         <f t="shared" si="4"/>
@@ -4933,15 +4951,15 @@
       </c>
       <c r="J7" s="22">
         <f>SUM(J2:J6)</f>
-        <v>17.483333333333334</v>
+        <v>33.049999999999997</v>
       </c>
       <c r="K7" s="25">
         <f>IF(SUM(K2:K6) &lt;&gt; 0, ((60*5) - SUM(K2:K6)) / 60, 0)</f>
-        <v>4.2666666666666666</v>
+        <v>2.75</v>
       </c>
       <c r="L7" s="34">
         <f>IF(SUM(L2:L6) &lt;&gt; 0, (SUM(L2:L6)/ 60), 0) * -1</f>
-        <v>0.41666666666666524</v>
+        <v>1.0999999999999972</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="24" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -4953,7 +4971,7 @@
       </c>
       <c r="J9" s="25">
         <f>40-J7</f>
-        <v>22.516666666666666</v>
+        <v>6.9500000000000028</v>
       </c>
       <c r="K9" s="26"/>
     </row>

</xml_diff>